<commit_message>
recactorisation code et création nouvlle fichier
</commit_message>
<xml_diff>
--- a/employes.xlsx
+++ b/employes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\developpeur1\PycharmProjects\Evaluation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D175EDCC-23F5-4126-9213-C0AF0CFBCD48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AA86E91-4DE3-41F1-987F-C68262BDCF4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-990" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="968" uniqueCount="668">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="967" uniqueCount="667">
   <si>
     <t>Matricule</t>
   </si>
@@ -1629,9 +1629,6 @@
   </si>
   <si>
     <t>6417</t>
-  </si>
-  <si>
-    <t>6420</t>
   </si>
   <si>
     <t>6567</t>
@@ -2456,7 +2453,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr codeName="Feuil1"/>
+  <sheetPr codeName="Feuil1" filterMode="1"/>
   <dimension ref="A1:F244"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2490,7 +2487,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>25</v>
@@ -2499,14 +2496,14 @@
         <v>264</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="E2" s="4">
         <v>976</v>
       </c>
       <c r="F2" s="4"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>454</v>
       </c>
@@ -2517,16 +2514,16 @@
         <v>280</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="E3" s="4">
         <v>976</v>
       </c>
       <c r="F3" s="4"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>133</v>
@@ -2535,16 +2532,16 @@
         <v>336</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="E4" s="4">
         <v>976</v>
       </c>
       <c r="F4" s="4"/>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>145</v>
@@ -2553,16 +2550,16 @@
         <v>345</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="E5" s="4">
         <v>976</v>
       </c>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>146</v>
@@ -2571,16 +2568,16 @@
         <v>346</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="E6" s="4">
         <v>976</v>
       </c>
       <c r="F6" s="4"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>148</v>
@@ -2589,16 +2586,16 @@
         <v>348</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="E7" s="4">
         <v>976</v>
       </c>
       <c r="F7" s="4"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="B8" t="s">
         <v>155</v>
@@ -2607,15 +2604,15 @@
         <v>348</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="E8" s="4">
         <v>976</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="B9" t="s">
         <v>196</v>
@@ -2624,15 +2621,15 @@
         <v>383</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="E9" s="4">
         <v>976</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="B10" t="s">
         <v>213</v>
@@ -2641,15 +2638,15 @@
         <v>395</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="E10" s="4">
         <v>976</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="B11" t="s">
         <v>221</v>
@@ -2658,7 +2655,7 @@
         <v>383</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="E11" s="4">
         <v>976</v>
@@ -2675,13 +2672,13 @@
         <v>278</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="E12">
         <v>1489</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>481</v>
       </c>
@@ -2692,13 +2689,13 @@
         <v>300</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="E13">
         <v>1489</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>7754</v>
       </c>
@@ -2709,15 +2706,15 @@
         <v>350</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="E14">
         <v>1489</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="B15" t="s">
         <v>167</v>
@@ -2726,15 +2723,15 @@
         <v>362</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="E15">
         <v>1489</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="B16" t="s">
         <v>172</v>
@@ -2743,15 +2740,15 @@
         <v>367</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="E16">
         <v>1489</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="B17" t="s">
         <v>192</v>
@@ -2760,15 +2757,15 @@
         <v>380</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="E17">
         <v>1489</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="B18" t="s">
         <v>243</v>
@@ -2777,15 +2774,15 @@
         <v>413</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="E18">
         <v>3507</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="B19" t="s">
         <v>246</v>
@@ -2794,15 +2791,15 @@
         <v>390</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="E19">
         <v>3507</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="B20" t="s">
         <v>247</v>
@@ -2811,13 +2808,13 @@
         <v>414</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="E20">
         <v>3507</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>3507</v>
       </c>
@@ -2828,13 +2825,13 @@
         <v>305</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="E21">
         <v>3507</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>502</v>
       </c>
@@ -2845,13 +2842,13 @@
         <v>308</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="E22">
         <v>3507</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>520</v>
       </c>
@@ -2862,7 +2859,7 @@
         <v>320</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="E23">
         <v>3507</v>
@@ -2879,15 +2876,15 @@
         <v>353</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="E24">
         <v>7867</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="B25" t="s">
         <v>169</v>
@@ -2896,15 +2893,15 @@
         <v>364</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="E25">
         <v>7867</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="B26" t="s">
         <v>176</v>
@@ -2913,15 +2910,15 @@
         <v>370</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="E26">
         <v>7867</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="B27" t="s">
         <v>200</v>
@@ -2930,15 +2927,15 @@
         <v>386</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="E27">
         <v>7867</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="B28" t="s">
         <v>205</v>
@@ -2947,15 +2944,15 @@
         <v>390</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="E28">
         <v>7867</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="B29" t="s">
         <v>222</v>
@@ -2964,13 +2961,13 @@
         <v>401</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="E29">
         <v>7867</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>509</v>
       </c>
@@ -2981,7 +2978,7 @@
         <v>313</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="E30">
         <v>4598</v>
@@ -2998,13 +2995,13 @@
         <v>314</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="E31">
         <v>4598</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>523</v>
       </c>
@@ -3015,13 +3012,13 @@
         <v>324</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="E32">
         <v>4598</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>528</v>
       </c>
@@ -3032,7 +3029,7 @@
         <v>327</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="E33">
         <v>4598</v>
@@ -3040,7 +3037,7 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="B34" t="s">
         <v>140</v>
@@ -3049,15 +3046,15 @@
         <v>340</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="E34">
         <v>4598</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="B35" t="s">
         <v>199</v>
@@ -3066,15 +3063,15 @@
         <v>385</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="E35">
         <v>4598</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="B36" t="s">
         <v>212</v>
@@ -3083,15 +3080,15 @@
         <v>394</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="E36">
         <v>4598</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="B37" t="s">
         <v>214</v>
@@ -3100,15 +3097,15 @@
         <v>396</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="E37">
         <v>4598</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="B38" t="s">
         <v>223</v>
@@ -3117,15 +3114,15 @@
         <v>402</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="E38">
         <v>4598</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="B39" s="6" t="s">
         <v>240</v>
@@ -3134,14 +3131,14 @@
         <v>412</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
       <c r="E39">
         <v>4598</v>
       </c>
       <c r="F39" s="6"/>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>527</v>
       </c>
@@ -3152,15 +3149,15 @@
         <v>326</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="E40">
         <v>6661</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="B41" t="s">
         <v>128</v>
@@ -3169,13 +3166,13 @@
         <v>331</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="E41">
         <v>6661</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>473</v>
       </c>
@@ -3186,15 +3183,15 @@
         <v>295</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="E42">
         <v>6661</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="B43" t="s">
         <v>186</v>
@@ -3203,13 +3200,13 @@
         <v>376</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="E43">
         <v>6661</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>426</v>
       </c>
@@ -3220,13 +3217,13 @@
         <v>258</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="E44">
         <v>6661</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>439</v>
       </c>
@@ -3237,13 +3234,13 @@
         <v>268</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="E45">
         <v>6661</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>449</v>
       </c>
@@ -3254,13 +3251,13 @@
         <v>277</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="E46">
         <v>6661</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>479</v>
       </c>
@@ -3271,15 +3268,15 @@
         <v>258</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="E47">
         <v>6661</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="B48" t="s">
         <v>129</v>
@@ -3288,13 +3285,13 @@
         <v>332</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="E48">
         <v>6661</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="2">
         <v>6661</v>
       </c>
@@ -3305,15 +3302,15 @@
         <v>334</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="E49">
         <v>6661</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="B50" t="s">
         <v>193</v>
@@ -3322,15 +3319,15 @@
         <v>381</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="E50">
         <v>6661</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="B51" t="s">
         <v>195</v>
@@ -3339,15 +3336,15 @@
         <v>382</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="E51">
         <v>6661</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="B52" t="s">
         <v>217</v>
@@ -3356,13 +3353,13 @@
         <v>399</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="E52">
         <v>6661</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>478</v>
       </c>
@@ -3373,13 +3370,13 @@
         <v>299</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="E53">
         <v>7266</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>518</v>
       </c>
@@ -3390,15 +3387,15 @@
         <v>319</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="E54">
         <v>7266</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B55" t="s">
         <v>126</v>
@@ -3407,7 +3404,7 @@
         <v>330</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="E55">
         <v>7266</v>
@@ -3424,15 +3421,15 @@
         <v>338</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="E56">
         <v>7266</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="B57" t="s">
         <v>144</v>
@@ -3441,15 +3438,15 @@
         <v>344</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="E57">
         <v>7266</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="B58" t="s">
         <v>156</v>
@@ -3458,15 +3455,15 @@
         <v>352</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="E58">
         <v>7266</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="B59" t="s">
         <v>159</v>
@@ -3475,15 +3472,15 @@
         <v>355</v>
       </c>
       <c r="D59" s="4" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="E59">
         <v>7266</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B60" t="s">
         <v>204</v>
@@ -3492,15 +3489,15 @@
         <v>389</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="E60">
         <v>7266</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="B61" t="s">
         <v>216</v>
@@ -3509,15 +3506,15 @@
         <v>398</v>
       </c>
       <c r="D61" s="4" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
       <c r="E61">
         <v>7266</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="B62" t="s">
         <v>244</v>
@@ -3526,12 +3523,12 @@
         <v>384</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="B63" t="s">
         <v>245</v>
@@ -3540,10 +3537,10 @@
         <v>384</v>
       </c>
       <c r="D63" s="4" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>446</v>
       </c>
@@ -3554,7 +3551,7 @@
         <v>274</v>
       </c>
       <c r="D64" s="4" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
@@ -3568,12 +3565,12 @@
         <v>322</v>
       </c>
       <c r="D65" s="4" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="B66" t="s">
         <v>160</v>
@@ -3582,12 +3579,12 @@
         <v>356</v>
       </c>
       <c r="D66" s="4" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="B67" t="s">
         <v>197</v>
@@ -3596,12 +3593,12 @@
         <v>384</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="B68" t="s">
         <v>218</v>
@@ -3610,12 +3607,12 @@
         <v>400</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="B69" t="s">
         <v>219</v>
@@ -3624,12 +3621,12 @@
         <v>384</v>
       </c>
       <c r="D69" s="4" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="B70" t="s">
         <v>220</v>
@@ -3638,12 +3635,12 @@
         <v>384</v>
       </c>
       <c r="D70" s="4" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="B71" t="s">
         <v>232</v>
@@ -3652,12 +3649,12 @@
         <v>384</v>
       </c>
       <c r="D71" s="4" t="s">
-        <v>658</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="5" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="B72" s="6" t="s">
         <v>241</v>
@@ -3666,7 +3663,7 @@
         <v>384</v>
       </c>
       <c r="D72" s="4" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="E72" s="6"/>
       <c r="F72" s="6"/>
@@ -3682,12 +3679,12 @@
         <v>316</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>665</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="B74" t="s">
         <v>139</v>
@@ -3696,12 +3693,12 @@
         <v>339</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>665</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="B75" t="s">
         <v>142</v>
@@ -3710,12 +3707,12 @@
         <v>342</v>
       </c>
       <c r="D75" s="4" t="s">
-        <v>665</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="B76" t="s">
         <v>147</v>
@@ -3724,12 +3721,12 @@
         <v>347</v>
       </c>
       <c r="D76" s="4" t="s">
-        <v>665</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="B77" t="s">
         <v>181</v>
@@ -3738,12 +3735,12 @@
         <v>373</v>
       </c>
       <c r="D77" s="4" t="s">
-        <v>665</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="B78" t="s">
         <v>201</v>
@@ -3752,12 +3749,12 @@
         <v>387</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>665</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="B79" t="s">
         <v>235</v>
@@ -3766,10 +3763,10 @@
         <v>342</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>665</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="9" t="s">
         <v>416</v>
       </c>
@@ -3780,12 +3777,12 @@
         <v>249</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="E80" s="11"/>
       <c r="F80" s="10"/>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="8" t="s">
         <v>417</v>
       </c>
@@ -3796,12 +3793,12 @@
         <v>250</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="E81" s="11"/>
       <c r="F81" s="10"/>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" s="8" t="s">
         <v>419</v>
       </c>
@@ -3812,12 +3809,12 @@
         <v>252</v>
       </c>
       <c r="D82" s="4" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="E82" s="11"/>
       <c r="F82" s="10"/>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" s="8" t="s">
         <v>420</v>
       </c>
@@ -3828,12 +3825,12 @@
         <v>253</v>
       </c>
       <c r="D83" s="4" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="E83" s="11"/>
       <c r="F83" s="10"/>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="10" t="s">
         <v>421</v>
       </c>
@@ -3844,12 +3841,12 @@
         <v>249</v>
       </c>
       <c r="D84" s="4" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="E84" s="11"/>
       <c r="F84" s="10"/>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
         <v>427</v>
       </c>
@@ -3860,10 +3857,10 @@
         <v>250</v>
       </c>
       <c r="D85" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
         <v>428</v>
       </c>
@@ -3874,10 +3871,10 @@
         <v>259</v>
       </c>
       <c r="D86" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
         <v>431</v>
       </c>
@@ -3888,10 +3885,10 @@
         <v>262</v>
       </c>
       <c r="D87" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
         <v>433</v>
       </c>
@@ -3902,10 +3899,10 @@
         <v>249</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
         <v>434</v>
       </c>
@@ -3916,10 +3913,10 @@
         <v>250</v>
       </c>
       <c r="D89" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
         <v>435</v>
       </c>
@@ -3930,12 +3927,12 @@
         <v>249</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="B91" t="s">
         <v>248</v>
@@ -3944,10 +3941,10 @@
         <v>415</v>
       </c>
       <c r="D91" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
         <v>436</v>
       </c>
@@ -3958,10 +3955,10 @@
         <v>265</v>
       </c>
       <c r="D92" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
         <v>437</v>
       </c>
@@ -3972,10 +3969,10 @@
         <v>266</v>
       </c>
       <c r="D93" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
         <v>441</v>
       </c>
@@ -3986,10 +3983,10 @@
         <v>270</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
         <v>442</v>
       </c>
@@ -4000,10 +3997,10 @@
         <v>271</v>
       </c>
       <c r="D95" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
         <v>443</v>
       </c>
@@ -4014,10 +4011,10 @@
         <v>272</v>
       </c>
       <c r="D96" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
         <v>445</v>
       </c>
@@ -4028,10 +4025,10 @@
         <v>271</v>
       </c>
       <c r="D97" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
         <v>448</v>
       </c>
@@ -4042,10 +4039,10 @@
         <v>276</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
         <v>450</v>
       </c>
@@ -4056,10 +4053,10 @@
         <v>265</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
         <v>451</v>
       </c>
@@ -4070,10 +4067,10 @@
         <v>265</v>
       </c>
       <c r="D100" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
         <v>452</v>
       </c>
@@ -4084,10 +4081,10 @@
         <v>279</v>
       </c>
       <c r="D101" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
         <v>453</v>
       </c>
@@ -4098,10 +4095,10 @@
         <v>265</v>
       </c>
       <c r="D102" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
         <v>455</v>
       </c>
@@ -4112,10 +4109,10 @@
         <v>281</v>
       </c>
       <c r="D103" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
         <v>456</v>
       </c>
@@ -4126,10 +4123,10 @@
         <v>265</v>
       </c>
       <c r="D104" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
         <v>457</v>
       </c>
@@ -4140,7 +4137,7 @@
         <v>250</v>
       </c>
       <c r="D105" s="4" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
@@ -4154,10 +4151,10 @@
         <v>283</v>
       </c>
       <c r="D106" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
         <v>463</v>
       </c>
@@ -4168,10 +4165,10 @@
         <v>265</v>
       </c>
       <c r="D107" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
         <v>467</v>
       </c>
@@ -4182,10 +4179,10 @@
         <v>290</v>
       </c>
       <c r="D108" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
         <v>470</v>
       </c>
@@ -4196,10 +4193,10 @@
         <v>293</v>
       </c>
       <c r="D109" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
         <v>471</v>
       </c>
@@ -4210,10 +4207,10 @@
         <v>265</v>
       </c>
       <c r="D110" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
         <v>474</v>
       </c>
@@ -4224,10 +4221,10 @@
         <v>296</v>
       </c>
       <c r="D111" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
         <v>475</v>
       </c>
@@ -4238,10 +4235,10 @@
         <v>297</v>
       </c>
       <c r="D112" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
         <v>477</v>
       </c>
@@ -4252,10 +4249,10 @@
         <v>265</v>
       </c>
       <c r="D113" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
         <v>480</v>
       </c>
@@ -4266,10 +4263,10 @@
         <v>253</v>
       </c>
       <c r="D114" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
         <v>486</v>
       </c>
@@ -4280,10 +4277,10 @@
         <v>265</v>
       </c>
       <c r="D115" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
         <v>488</v>
       </c>
@@ -4294,10 +4291,10 @@
         <v>250</v>
       </c>
       <c r="D116" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
         <v>489</v>
       </c>
@@ -4308,10 +4305,10 @@
         <v>304</v>
       </c>
       <c r="D117" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
         <v>490</v>
       </c>
@@ -4322,10 +4319,10 @@
         <v>249</v>
       </c>
       <c r="D118" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
         <v>491</v>
       </c>
@@ -4336,10 +4333,10 @@
         <v>250</v>
       </c>
       <c r="D119" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
         <v>492</v>
       </c>
@@ -4350,10 +4347,10 @@
         <v>250</v>
       </c>
       <c r="D120" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
         <v>493</v>
       </c>
@@ -4364,10 +4361,10 @@
         <v>249</v>
       </c>
       <c r="D121" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
         <v>494</v>
       </c>
@@ -4378,10 +4375,10 @@
         <v>265</v>
       </c>
       <c r="D122" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
         <v>495</v>
       </c>
@@ -4392,10 +4389,10 @@
         <v>290</v>
       </c>
       <c r="D123" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
         <v>499</v>
       </c>
@@ -4406,10 +4403,10 @@
         <v>265</v>
       </c>
       <c r="D124" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
         <v>500</v>
       </c>
@@ -4420,10 +4417,10 @@
         <v>265</v>
       </c>
       <c r="D125" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
         <v>503</v>
       </c>
@@ -4434,10 +4431,10 @@
         <v>265</v>
       </c>
       <c r="D126" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
         <v>511</v>
       </c>
@@ -4448,10 +4445,10 @@
         <v>265</v>
       </c>
       <c r="D127" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
         <v>516</v>
       </c>
@@ -4462,12 +4459,12 @@
         <v>265</v>
       </c>
       <c r="D128" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B129" t="s">
         <v>127</v>
@@ -4476,12 +4473,12 @@
         <v>265</v>
       </c>
       <c r="D129" s="4" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="B130" t="s">
         <v>141</v>
@@ -4490,12 +4487,12 @@
         <v>341</v>
       </c>
       <c r="D130" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="B131" t="s">
         <v>165</v>
@@ -4504,10 +4501,10 @@
         <v>360</v>
       </c>
       <c r="D131" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A132" s="2">
         <v>8063</v>
       </c>
@@ -4518,12 +4515,12 @@
         <v>365</v>
       </c>
       <c r="D132" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="B133" t="s">
         <v>175</v>
@@ -4532,12 +4529,12 @@
         <v>369</v>
       </c>
       <c r="D133" s="4" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="B134" t="s">
         <v>185</v>
@@ -4546,12 +4543,12 @@
         <v>375</v>
       </c>
       <c r="D134" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="B135" t="s">
         <v>188</v>
@@ -4560,12 +4557,12 @@
         <v>265</v>
       </c>
       <c r="D135" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
       <c r="B136" t="s">
         <v>189</v>
@@ -4574,12 +4571,12 @@
         <v>378</v>
       </c>
       <c r="D136" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="B137" t="s">
         <v>225</v>
@@ -4588,12 +4585,12 @@
         <v>403</v>
       </c>
       <c r="D137" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B138" t="s">
         <v>227</v>
@@ -4602,12 +4599,12 @@
         <v>405</v>
       </c>
       <c r="D138" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="B139" t="s">
         <v>231</v>
@@ -4616,12 +4613,12 @@
         <v>391</v>
       </c>
       <c r="D139" s="4" t="s">
-        <v>649</v>
-      </c>
-    </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A140" s="5" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="B140" s="6" t="s">
         <v>237</v>
@@ -4630,12 +4627,12 @@
         <v>409</v>
       </c>
       <c r="D140" s="4" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="E140" s="6"/>
       <c r="F140" s="6"/>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
         <v>512</v>
       </c>
@@ -4646,13 +4643,13 @@
         <v>315</v>
       </c>
       <c r="D141" s="4" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="E141">
         <v>9313</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
         <v>517</v>
       </c>
@@ -4663,15 +4660,15 @@
         <v>318</v>
       </c>
       <c r="D142" s="4" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="E142">
         <v>9313</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="B143" t="s">
         <v>191</v>
@@ -4680,7 +4677,7 @@
         <v>379</v>
       </c>
       <c r="D143" s="4" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="E143">
         <v>9313</v>
@@ -4697,15 +4694,15 @@
         <v>388</v>
       </c>
       <c r="D144" s="4" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="E144">
-        <v>9313</v>
-      </c>
-    </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
+        <v>6420</v>
+      </c>
+    </row>
+    <row r="145" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A145" s="5" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="B145" s="6" t="s">
         <v>242</v>
@@ -4714,7 +4711,7 @@
         <v>379</v>
       </c>
       <c r="D145" s="4" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="E145">
         <v>9313</v>
@@ -4732,7 +4729,7 @@
         <v>255</v>
       </c>
       <c r="D146" s="4" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.25">
@@ -4746,7 +4743,7 @@
         <v>256</v>
       </c>
       <c r="D147" s="4" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.25">
@@ -4760,12 +4757,12 @@
         <v>263</v>
       </c>
       <c r="D148" s="4" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A149" s="2" t="s">
-        <v>530</v>
+      <c r="A149" s="2">
+        <v>6420</v>
       </c>
       <c r="B149" t="s">
         <v>125</v>
@@ -4774,12 +4771,12 @@
         <v>329</v>
       </c>
       <c r="D149" s="4" t="s">
-        <v>651</v>
-      </c>
-    </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="B150" t="s">
         <v>158</v>
@@ -4788,12 +4785,12 @@
         <v>354</v>
       </c>
       <c r="D150" s="4" t="s">
-        <v>651</v>
-      </c>
-    </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.25">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="B151" t="s">
         <v>228</v>
@@ -4802,12 +4799,12 @@
         <v>406</v>
       </c>
       <c r="D151" s="4" t="s">
-        <v>651</v>
-      </c>
-    </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="152" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="B152" t="s">
         <v>233</v>
@@ -4816,12 +4813,12 @@
         <v>407</v>
       </c>
       <c r="D152" s="4" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="B153" t="s">
         <v>236</v>
@@ -4830,10 +4827,10 @@
         <v>408</v>
       </c>
       <c r="D153" s="4" t="s">
-        <v>651</v>
-      </c>
-    </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="154" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
         <v>429</v>
       </c>
@@ -4844,10 +4841,10 @@
         <v>260</v>
       </c>
       <c r="D154" s="4" t="s">
-        <v>655</v>
-      </c>
-    </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.25">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="155" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
         <v>430</v>
       </c>
@@ -4858,10 +4855,10 @@
         <v>261</v>
       </c>
       <c r="D155" s="4" t="s">
-        <v>655</v>
-      </c>
-    </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.25">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="156" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
         <v>462</v>
       </c>
@@ -4872,10 +4869,10 @@
         <v>286</v>
       </c>
       <c r="D156" s="4" t="s">
-        <v>655</v>
-      </c>
-    </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.25">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="157" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
         <v>465</v>
       </c>
@@ -4886,10 +4883,10 @@
         <v>288</v>
       </c>
       <c r="D157" s="4" t="s">
-        <v>655</v>
-      </c>
-    </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.25">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="158" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
         <v>466</v>
       </c>
@@ -4900,10 +4897,10 @@
         <v>289</v>
       </c>
       <c r="D158" s="4" t="s">
-        <v>655</v>
-      </c>
-    </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.25">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="159" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
         <v>469</v>
       </c>
@@ -4914,10 +4911,10 @@
         <v>292</v>
       </c>
       <c r="D159" s="4" t="s">
-        <v>655</v>
-      </c>
-    </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.25">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="160" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
         <v>482</v>
       </c>
@@ -4928,10 +4925,10 @@
         <v>288</v>
       </c>
       <c r="D160" s="4" t="s">
-        <v>655</v>
-      </c>
-    </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="161" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
         <v>484</v>
       </c>
@@ -4942,10 +4939,10 @@
         <v>288</v>
       </c>
       <c r="D161" s="4" t="s">
-        <v>655</v>
-      </c>
-    </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="162" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
         <v>487</v>
       </c>
@@ -4956,7 +4953,7 @@
         <v>303</v>
       </c>
       <c r="D162" s="4" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
@@ -4970,10 +4967,10 @@
         <v>306</v>
       </c>
       <c r="D163" s="4" t="s">
-        <v>655</v>
-      </c>
-    </row>
-    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="164" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A164" s="2" t="s">
         <v>497</v>
       </c>
@@ -4984,10 +4981,10 @@
         <v>260</v>
       </c>
       <c r="D164" s="4" t="s">
-        <v>655</v>
-      </c>
-    </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="165" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A165" s="2" t="s">
         <v>498</v>
       </c>
@@ -4998,10 +4995,10 @@
         <v>288</v>
       </c>
       <c r="D165" s="4" t="s">
-        <v>655</v>
-      </c>
-    </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="166" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A166" s="2" t="s">
         <v>505</v>
       </c>
@@ -5012,10 +5009,10 @@
         <v>309</v>
       </c>
       <c r="D166" s="4" t="s">
-        <v>655</v>
-      </c>
-    </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="167" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A167" s="2" t="s">
         <v>510</v>
       </c>
@@ -5026,10 +5023,10 @@
         <v>260</v>
       </c>
       <c r="D167" s="4" t="s">
-        <v>655</v>
-      </c>
-    </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="168" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A168" s="2" t="s">
         <v>514</v>
       </c>
@@ -5040,12 +5037,12 @@
         <v>292</v>
       </c>
       <c r="D168" s="4" t="s">
-        <v>655</v>
-      </c>
-    </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="169" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A169" s="2" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="B169" t="s">
         <v>135</v>
@@ -5054,12 +5051,12 @@
         <v>292</v>
       </c>
       <c r="D169" s="4" t="s">
-        <v>655</v>
-      </c>
-    </row>
-    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="170" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A170" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="B170" t="s">
         <v>161</v>
@@ -5068,10 +5065,10 @@
         <v>357</v>
       </c>
       <c r="D170" s="4" t="s">
-        <v>655</v>
-      </c>
-    </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="171" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A171" s="2" t="s">
         <v>438</v>
       </c>
@@ -5082,7 +5079,7 @@
         <v>267</v>
       </c>
       <c r="D171" s="4" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.25">
@@ -5096,10 +5093,10 @@
         <v>294</v>
       </c>
       <c r="D172" s="4" t="s">
-        <v>656</v>
-      </c>
-    </row>
-    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="173" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A173" s="2" t="s">
         <v>501</v>
       </c>
@@ -5110,10 +5107,10 @@
         <v>307</v>
       </c>
       <c r="D173" s="4" t="s">
-        <v>656</v>
-      </c>
-    </row>
-    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="174" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A174" s="2" t="s">
         <v>526</v>
       </c>
@@ -5124,12 +5121,12 @@
         <v>325</v>
       </c>
       <c r="D174" s="4" t="s">
-        <v>656</v>
-      </c>
-    </row>
-    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="175" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A175" s="2" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="B175" t="s">
         <v>153</v>
@@ -5138,12 +5135,12 @@
         <v>351</v>
       </c>
       <c r="D175" s="4" t="s">
-        <v>656</v>
-      </c>
-    </row>
-    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="176" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A176" s="2" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="B176" t="s">
         <v>182</v>
@@ -5152,12 +5149,12 @@
         <v>267</v>
       </c>
       <c r="D176" s="4" t="s">
-        <v>656</v>
-      </c>
-    </row>
-    <row r="177" spans="1:4" x14ac:dyDescent="0.25">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="177" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="B177" t="s">
         <v>194</v>
@@ -5166,12 +5163,12 @@
         <v>325</v>
       </c>
       <c r="D177" s="4" t="s">
-        <v>656</v>
-      </c>
-    </row>
-    <row r="178" spans="1:4" x14ac:dyDescent="0.25">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="178" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A178" s="2" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="B178" t="s">
         <v>203</v>
@@ -5180,12 +5177,12 @@
         <v>325</v>
       </c>
       <c r="D178" s="4" t="s">
-        <v>656</v>
-      </c>
-    </row>
-    <row r="179" spans="1:4" x14ac:dyDescent="0.25">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="179" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A179" s="2" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="B179" t="s">
         <v>206</v>
@@ -5194,12 +5191,12 @@
         <v>325</v>
       </c>
       <c r="D179" s="4" t="s">
-        <v>656</v>
-      </c>
-    </row>
-    <row r="180" spans="1:4" x14ac:dyDescent="0.25">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="180" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A180" s="2" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B180" t="s">
         <v>207</v>
@@ -5208,12 +5205,12 @@
         <v>325</v>
       </c>
       <c r="D180" s="4" t="s">
-        <v>656</v>
-      </c>
-    </row>
-    <row r="181" spans="1:4" x14ac:dyDescent="0.25">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="181" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A181" s="2" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="B181" t="s">
         <v>211</v>
@@ -5222,10 +5219,10 @@
         <v>325</v>
       </c>
       <c r="D181" s="4" t="s">
-        <v>656</v>
-      </c>
-    </row>
-    <row r="182" spans="1:4" x14ac:dyDescent="0.25">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="182" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A182" s="2" t="s">
         <v>425</v>
       </c>
@@ -5236,10 +5233,10 @@
         <v>257</v>
       </c>
       <c r="D182" s="4" t="s">
-        <v>652</v>
-      </c>
-    </row>
-    <row r="183" spans="1:4" x14ac:dyDescent="0.25">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="183" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A183" s="2" t="s">
         <v>515</v>
       </c>
@@ -5250,10 +5247,10 @@
         <v>317</v>
       </c>
       <c r="D183" s="4" t="s">
-        <v>652</v>
-      </c>
-    </row>
-    <row r="184" spans="1:4" x14ac:dyDescent="0.25">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="184" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A184" s="2" t="s">
         <v>519</v>
       </c>
@@ -5264,12 +5261,12 @@
         <v>317</v>
       </c>
       <c r="D184" s="4" t="s">
-        <v>652</v>
-      </c>
-    </row>
-    <row r="185" spans="1:4" x14ac:dyDescent="0.25">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="185" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A185" s="2" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="B185" t="s">
         <v>132</v>
@@ -5278,12 +5275,12 @@
         <v>335</v>
       </c>
       <c r="D185" s="4" t="s">
-        <v>652</v>
-      </c>
-    </row>
-    <row r="186" spans="1:4" x14ac:dyDescent="0.25">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="186" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A186" s="2" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="B186" t="s">
         <v>138</v>
@@ -5292,12 +5289,12 @@
         <v>317</v>
       </c>
       <c r="D186" s="4" t="s">
-        <v>652</v>
-      </c>
-    </row>
-    <row r="187" spans="1:4" x14ac:dyDescent="0.25">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="187" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A187" s="2" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="B187" t="s">
         <v>151</v>
@@ -5306,12 +5303,12 @@
         <v>317</v>
       </c>
       <c r="D187" s="4" t="s">
-        <v>652</v>
-      </c>
-    </row>
-    <row r="188" spans="1:4" x14ac:dyDescent="0.25">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="188" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A188" s="2" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="B188" t="s">
         <v>152</v>
@@ -5320,12 +5317,12 @@
         <v>317</v>
       </c>
       <c r="D188" s="4" t="s">
-        <v>652</v>
-      </c>
-    </row>
-    <row r="189" spans="1:4" x14ac:dyDescent="0.25">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="189" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A189" s="2" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="B189" t="s">
         <v>166</v>
@@ -5334,12 +5331,12 @@
         <v>361</v>
       </c>
       <c r="D189" s="4" t="s">
-        <v>652</v>
-      </c>
-    </row>
-    <row r="190" spans="1:4" x14ac:dyDescent="0.25">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="190" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A190" s="2" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="B190" t="s">
         <v>168</v>
@@ -5348,12 +5345,12 @@
         <v>363</v>
       </c>
       <c r="D190" s="4" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
     </row>
     <row r="191" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A191" s="2" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="B191" t="s">
         <v>179</v>
@@ -5362,12 +5359,12 @@
         <v>371</v>
       </c>
       <c r="D191" s="4" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
     </row>
     <row r="192" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A192" s="2" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="B192" t="s">
         <v>180</v>
@@ -5376,12 +5373,12 @@
         <v>372</v>
       </c>
       <c r="D192" s="4" t="s">
-        <v>652</v>
-      </c>
-    </row>
-    <row r="193" spans="1:6" x14ac:dyDescent="0.25">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="193" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A193" s="2" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="B193" t="s">
         <v>187</v>
@@ -5390,12 +5387,12 @@
         <v>377</v>
       </c>
       <c r="D193" s="4" t="s">
-        <v>652</v>
-      </c>
-    </row>
-    <row r="194" spans="1:6" x14ac:dyDescent="0.25">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="194" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A194" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="B194" t="s">
         <v>190</v>
@@ -5404,12 +5401,12 @@
         <v>335</v>
       </c>
       <c r="D194" s="4" t="s">
-        <v>652</v>
-      </c>
-    </row>
-    <row r="195" spans="1:6" x14ac:dyDescent="0.25">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="195" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A195" s="2" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="B195" t="s">
         <v>198</v>
@@ -5418,12 +5415,12 @@
         <v>317</v>
       </c>
       <c r="D195" s="4" t="s">
-        <v>652</v>
-      </c>
-    </row>
-    <row r="196" spans="1:6" x14ac:dyDescent="0.25">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="196" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A196" s="2" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B196" t="s">
         <v>215</v>
@@ -5432,12 +5429,12 @@
         <v>397</v>
       </c>
       <c r="D196" s="4" t="s">
-        <v>652</v>
-      </c>
-    </row>
-    <row r="197" spans="1:6" x14ac:dyDescent="0.25">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="197" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A197" s="2" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B197" t="s">
         <v>224</v>
@@ -5446,12 +5443,12 @@
         <v>377</v>
       </c>
       <c r="D197" s="4" t="s">
-        <v>652</v>
-      </c>
-    </row>
-    <row r="198" spans="1:6" x14ac:dyDescent="0.25">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="198" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A198" s="2" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="B198" t="s">
         <v>229</v>
@@ -5460,12 +5457,12 @@
         <v>317</v>
       </c>
       <c r="D198" s="4" t="s">
-        <v>652</v>
-      </c>
-    </row>
-    <row r="199" spans="1:6" x14ac:dyDescent="0.25">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="199" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A199" s="2" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="B199" t="s">
         <v>234</v>
@@ -5474,12 +5471,12 @@
         <v>317</v>
       </c>
       <c r="D199" s="4" t="s">
-        <v>652</v>
-      </c>
-    </row>
-    <row r="200" spans="1:6" x14ac:dyDescent="0.25">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="200" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A200" s="5" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="B200" s="6" t="s">
         <v>239</v>
@@ -5488,12 +5485,12 @@
         <v>411</v>
       </c>
       <c r="D200" s="4" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="E200" s="6"/>
       <c r="F200" s="6"/>
     </row>
-    <row r="201" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A201" s="2" t="s">
         <v>476</v>
       </c>
@@ -5504,7 +5501,7 @@
         <v>298</v>
       </c>
       <c r="D201" s="4" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
     </row>
     <row r="202" spans="1:6" x14ac:dyDescent="0.25">
@@ -5518,12 +5515,12 @@
         <v>302</v>
       </c>
       <c r="D202" s="4" t="s">
-        <v>661</v>
-      </c>
-    </row>
-    <row r="203" spans="1:6" x14ac:dyDescent="0.25">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="203" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A203" s="5" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="B203" s="6" t="s">
         <v>238</v>
@@ -5532,12 +5529,12 @@
         <v>410</v>
       </c>
       <c r="D203" s="4" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="E203" s="6"/>
       <c r="F203" s="6"/>
     </row>
-    <row r="204" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A204" s="2" t="s">
         <v>422</v>
       </c>
@@ -5548,10 +5545,10 @@
         <v>254</v>
       </c>
       <c r="D204" s="4" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="205" spans="1:6" x14ac:dyDescent="0.25">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="205" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A205" s="2" t="s">
         <v>444</v>
       </c>
@@ -5562,10 +5559,10 @@
         <v>273</v>
       </c>
       <c r="D205" s="4" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="206" spans="1:6" x14ac:dyDescent="0.25">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="206" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A206" s="2" t="s">
         <v>447</v>
       </c>
@@ -5576,10 +5573,10 @@
         <v>275</v>
       </c>
       <c r="D206" s="4" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="207" spans="1:6" x14ac:dyDescent="0.25">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="207" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A207" s="2" t="s">
         <v>460</v>
       </c>
@@ -5590,10 +5587,10 @@
         <v>284</v>
       </c>
       <c r="D207" s="4" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="208" spans="1:6" x14ac:dyDescent="0.25">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="208" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A208" s="2" t="s">
         <v>464</v>
       </c>
@@ -5604,10 +5601,10 @@
         <v>287</v>
       </c>
       <c r="D208" s="4" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="209" spans="1:4" x14ac:dyDescent="0.25">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="209" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A209" s="2" t="s">
         <v>468</v>
       </c>
@@ -5618,10 +5615,10 @@
         <v>291</v>
       </c>
       <c r="D209" s="4" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="210" spans="1:4" x14ac:dyDescent="0.25">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="210" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A210" s="2" t="s">
         <v>483</v>
       </c>
@@ -5632,10 +5629,10 @@
         <v>301</v>
       </c>
       <c r="D210" s="4" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="211" spans="1:4" x14ac:dyDescent="0.25">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="211" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A211" s="2" t="s">
         <v>506</v>
       </c>
@@ -5646,10 +5643,10 @@
         <v>310</v>
       </c>
       <c r="D211" s="4" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="212" spans="1:4" x14ac:dyDescent="0.25">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="212" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A212" s="2" t="s">
         <v>521</v>
       </c>
@@ -5660,10 +5657,10 @@
         <v>321</v>
       </c>
       <c r="D212" s="4" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="213" spans="1:4" x14ac:dyDescent="0.25">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="213" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A213" s="2" t="s">
         <v>522</v>
       </c>
@@ -5674,10 +5671,10 @@
         <v>323</v>
       </c>
       <c r="D213" s="4" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="214" spans="1:4" x14ac:dyDescent="0.25">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="214" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A214" s="2" t="s">
         <v>524</v>
       </c>
@@ -5688,10 +5685,10 @@
         <v>275</v>
       </c>
       <c r="D214" s="4" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="215" spans="1:4" x14ac:dyDescent="0.25">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="215" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A215" s="2" t="s">
         <v>525</v>
       </c>
@@ -5702,12 +5699,12 @@
         <v>275</v>
       </c>
       <c r="D215" s="4" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="216" spans="1:4" x14ac:dyDescent="0.25">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="216" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A216" s="2" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="B216" t="s">
         <v>134</v>
@@ -5716,12 +5713,12 @@
         <v>321</v>
       </c>
       <c r="D216" s="4" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="217" spans="1:4" x14ac:dyDescent="0.25">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="217" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A217" s="2" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B217" t="s">
         <v>143</v>
@@ -5730,12 +5727,12 @@
         <v>343</v>
       </c>
       <c r="D217" s="4" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="218" spans="1:4" x14ac:dyDescent="0.25">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="218" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A218" s="2" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="B218" t="s">
         <v>149</v>
@@ -5744,12 +5741,12 @@
         <v>349</v>
       </c>
       <c r="D218" s="4" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="219" spans="1:4" x14ac:dyDescent="0.25">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="219" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A219" s="2" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="B219" t="s">
         <v>164</v>
@@ -5758,12 +5755,12 @@
         <v>321</v>
       </c>
       <c r="D219" s="4" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="220" spans="1:4" x14ac:dyDescent="0.25">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="220" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A220" s="2" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="B220" t="s">
         <v>171</v>
@@ -5772,12 +5769,12 @@
         <v>366</v>
       </c>
       <c r="D220" s="4" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="221" spans="1:4" x14ac:dyDescent="0.25">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="221" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A221" s="2" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="B221" t="s">
         <v>173</v>
@@ -5786,12 +5783,12 @@
         <v>368</v>
       </c>
       <c r="D221" s="4" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="222" spans="1:4" x14ac:dyDescent="0.25">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="222" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A222" s="2" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="B222" t="s">
         <v>174</v>
@@ -5800,12 +5797,12 @@
         <v>321</v>
       </c>
       <c r="D222" s="4" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="223" spans="1:4" x14ac:dyDescent="0.25">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="223" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A223" s="2" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="B223" t="s">
         <v>177</v>
@@ -5814,12 +5811,12 @@
         <v>301</v>
       </c>
       <c r="D223" s="4" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="224" spans="1:4" x14ac:dyDescent="0.25">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="224" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A224" s="2" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="B224" t="s">
         <v>178</v>
@@ -5828,12 +5825,12 @@
         <v>321</v>
       </c>
       <c r="D224" s="4" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="225" spans="1:6" x14ac:dyDescent="0.25">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="225" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A225" s="2" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B225" t="s">
         <v>208</v>
@@ -5842,12 +5839,12 @@
         <v>391</v>
       </c>
       <c r="D225" s="4" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="226" spans="1:6" x14ac:dyDescent="0.25">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="226" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A226" s="2" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="B226" t="s">
         <v>209</v>
@@ -5856,12 +5853,12 @@
         <v>392</v>
       </c>
       <c r="D226" s="4" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="227" spans="1:6" x14ac:dyDescent="0.25">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="227" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A227" s="2" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="B227" t="s">
         <v>210</v>
@@ -5870,12 +5867,12 @@
         <v>393</v>
       </c>
       <c r="D227" s="4" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="228" spans="1:6" x14ac:dyDescent="0.25">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="228" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A228" s="2" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="B228" t="s">
         <v>226</v>
@@ -5884,10 +5881,10 @@
         <v>404</v>
       </c>
       <c r="D228" s="4" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="229" spans="1:6" x14ac:dyDescent="0.25">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="229" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A229" s="8" t="s">
         <v>418</v>
       </c>
@@ -5898,12 +5895,12 @@
         <v>251</v>
       </c>
       <c r="D229" s="4" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="E229" s="11"/>
       <c r="F229" s="10"/>
     </row>
-    <row r="230" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A230" s="2" t="s">
         <v>440</v>
       </c>
@@ -5914,10 +5911,10 @@
         <v>269</v>
       </c>
       <c r="D230" s="4" t="s">
-        <v>648</v>
-      </c>
-    </row>
-    <row r="231" spans="1:6" x14ac:dyDescent="0.25">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="231" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A231" s="2" t="s">
         <v>458</v>
       </c>
@@ -5928,10 +5925,10 @@
         <v>282</v>
       </c>
       <c r="D231" s="4" t="s">
-        <v>648</v>
-      </c>
-    </row>
-    <row r="232" spans="1:6" x14ac:dyDescent="0.25">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="232" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A232" s="2" t="s">
         <v>461</v>
       </c>
@@ -5942,10 +5939,10 @@
         <v>285</v>
       </c>
       <c r="D232" s="4" t="s">
-        <v>648</v>
-      </c>
-    </row>
-    <row r="233" spans="1:6" x14ac:dyDescent="0.25">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="233" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A233" s="2" t="s">
         <v>504</v>
       </c>
@@ -5956,10 +5953,10 @@
         <v>282</v>
       </c>
       <c r="D233" s="4" t="s">
-        <v>648</v>
-      </c>
-    </row>
-    <row r="234" spans="1:6" x14ac:dyDescent="0.25">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="234" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A234" s="2" t="s">
         <v>507</v>
       </c>
@@ -5970,10 +5967,10 @@
         <v>311</v>
       </c>
       <c r="D234" s="4" t="s">
-        <v>648</v>
-      </c>
-    </row>
-    <row r="235" spans="1:6" x14ac:dyDescent="0.25">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="235" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A235" s="2" t="s">
         <v>508</v>
       </c>
@@ -5984,10 +5981,10 @@
         <v>312</v>
       </c>
       <c r="D235" s="4" t="s">
-        <v>648</v>
-      </c>
-    </row>
-    <row r="236" spans="1:6" x14ac:dyDescent="0.25">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="236" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A236" s="2" t="s">
         <v>529</v>
       </c>
@@ -5998,12 +5995,12 @@
         <v>328</v>
       </c>
       <c r="D236" s="4" t="s">
-        <v>648</v>
-      </c>
-    </row>
-    <row r="237" spans="1:6" x14ac:dyDescent="0.25">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="237" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A237" s="2" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B237" t="s">
         <v>130</v>
@@ -6012,12 +6009,12 @@
         <v>333</v>
       </c>
       <c r="D237" s="4" t="s">
-        <v>648</v>
-      </c>
-    </row>
-    <row r="238" spans="1:6" x14ac:dyDescent="0.25">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="238" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A238" s="2" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="B238" t="s">
         <v>136</v>
@@ -6026,12 +6023,12 @@
         <v>337</v>
       </c>
       <c r="D238" s="4" t="s">
-        <v>648</v>
-      </c>
-    </row>
-    <row r="239" spans="1:6" x14ac:dyDescent="0.25">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="239" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A239" s="2" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="B239" t="s">
         <v>154</v>
@@ -6040,12 +6037,12 @@
         <v>311</v>
       </c>
       <c r="D239" s="4" t="s">
-        <v>648</v>
-      </c>
-    </row>
-    <row r="240" spans="1:6" x14ac:dyDescent="0.25">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="240" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A240" s="2" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="B240" t="s">
         <v>162</v>
@@ -6054,12 +6051,12 @@
         <v>358</v>
       </c>
       <c r="D240" s="4" t="s">
-        <v>648</v>
-      </c>
-    </row>
-    <row r="241" spans="1:6" x14ac:dyDescent="0.25">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="241" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A241" s="2" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="B241" t="s">
         <v>163</v>
@@ -6068,12 +6065,12 @@
         <v>359</v>
       </c>
       <c r="D241" s="4" t="s">
-        <v>648</v>
-      </c>
-    </row>
-    <row r="242" spans="1:6" x14ac:dyDescent="0.25">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="242" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A242" s="5" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="B242" s="6" t="s">
         <v>183</v>
@@ -6082,14 +6079,14 @@
         <v>374</v>
       </c>
       <c r="D242" s="4" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="E242" s="6"/>
       <c r="F242" s="6"/>
     </row>
-    <row r="243" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A243" s="5" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="B243" s="6" t="s">
         <v>184</v>
@@ -6098,14 +6095,14 @@
         <v>374</v>
       </c>
       <c r="D243" s="4" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="E243" s="6"/>
       <c r="F243" s="6"/>
     </row>
-    <row r="244" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A244" s="2" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="B244" t="s">
         <v>230</v>
@@ -6114,11 +6111,37 @@
         <v>312</v>
       </c>
       <c r="D244" s="4" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:F244" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="ADJ DIRECTEUR QHSE"/>
+        <filter val="DIRECTEUR ADJ MAGASIN"/>
+        <filter val="DIRECTEUR GENERAL"/>
+        <filter val="DIRECTEUR GENERAL ADJ"/>
+        <filter val="DIRECTEUR INFORMATIQUE ET SI"/>
+        <filter val="DIRECTEUR PRODUCTION"/>
+        <filter val="DIRECTRICE ADJ DEV RH ET CENTR"/>
+        <filter val="DIRECTRICE ADJ ERP"/>
+        <filter val="DIRECTRICE ADJ GESCOM"/>
+        <filter val="DIRECTRICE ADJ LEAN"/>
+        <filter val="DIRECTRICE ADJ PROJETS INDUSTR"/>
+        <filter val="DIRECTRICE COMMERCIALE"/>
+        <filter val="DIRECTRICE COMMERCIALE ADJ"/>
+        <filter val="DIRECTRICE CONFORMITE DES PROC"/>
+        <filter val="DIRECTRICE CONSEILLER AUPRES D"/>
+        <filter val="DIRECTRICE DEV ET CDG"/>
+        <filter val="DIRECTRICE FINANCIER"/>
+        <filter val="DIRECTRICE PROD ADJ"/>
+        <filter val="DIRECTRICE QHSE"/>
+        <filter val="DIRECTRICE QUALITE PRODUIT"/>
+        <filter val="DIRECTRICE TRANSIT"/>
+        <filter val="PRESIDENT DIRECTEUR GENERAL"/>
+      </filters>
+    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F244">
       <sortCondition descending="1" ref="D1:D244"/>
     </sortState>

</xml_diff>